<commit_message>
Add optional chords to songs
</commit_message>
<xml_diff>
--- a/assets/modelo_importacao_musicas.xlsx
+++ b/assets/modelo_importacao_musicas.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Musicas" sheetId="1" r:id="R4a02058724a94796"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="2" r:id="R5ff9e26c02a44f9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Musicas" sheetId="1" r:id="R29c38e54fd6a43c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="2" r:id="R5e96a27f08b74bf5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37,7 +37,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -57,6 +57,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF7A5428"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF245C52"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -94,7 +99,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -149,6 +154,14 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -369,6 +382,17 @@
     <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="10" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="10" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="18" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="18" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="18" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -422,6 +446,39 @@
       </x:c>
       <x:c r="Q1" s="4" t="str">
         <x:v>ativa</x:v>
+      </x:c>
+      <x:c r="R1" s="29" t="str">
+        <x:v>cifra_refrao</x:v>
+      </x:c>
+      <x:c r="S1" s="29" t="str">
+        <x:v>cifra_1</x:v>
+      </x:c>
+      <x:c r="T1" s="29" t="str">
+        <x:v>cifra_2</x:v>
+      </x:c>
+      <x:c r="U1" s="29" t="str">
+        <x:v>cifra_3</x:v>
+      </x:c>
+      <x:c r="V1" s="29" t="str">
+        <x:v>cifra_4</x:v>
+      </x:c>
+      <x:c r="W1" s="29" t="str">
+        <x:v>cifra_5</x:v>
+      </x:c>
+      <x:c r="X1" s="29" t="str">
+        <x:v>cifra_6</x:v>
+      </x:c>
+      <x:c r="Y1" s="29" t="str">
+        <x:v>cifra_7</x:v>
+      </x:c>
+      <x:c r="Z1" s="29" t="str">
+        <x:v>cifra_8</x:v>
+      </x:c>
+      <x:c r="AA1" s="29" t="str">
+        <x:v>cifra_9</x:v>
+      </x:c>
+      <x:c r="AB1" s="29" t="str">
+        <x:v>cifra_10</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="76" customHeight="1">
@@ -463,6 +520,25 @@
       <x:c r="Q2" s="11" t="str">
         <x:v>sim</x:v>
       </x:c>
+      <x:c r="R2" s="30" t="str">
+        <x:v>G   D   A</x:v>
+      </x:c>
+      <x:c r="S2" s="30" t="str">
+        <x:v>D   A   Bm   G</x:v>
+      </x:c>
+      <x:c r="T2" s="30" t="str">
+        <x:v>G   D   A</x:v>
+      </x:c>
+      <x:c r="U2" s="30" t="str">
+        <x:v>Bm   G   D   A</x:v>
+      </x:c>
+      <x:c r="V2" s="30" t="str"/>
+      <x:c r="W2" s="30" t="str"/>
+      <x:c r="X2" s="30" t="str"/>
+      <x:c r="Y2" s="30" t="str"/>
+      <x:c r="Z2" s="30" t="str"/>
+      <x:c r="AA2" s="30" t="str"/>
+      <x:c r="AB2" s="30" t="str"/>
     </x:row>
     <x:row r="3" ht="76" customHeight="1">
       <x:c r="A3" s="12" t="str">
@@ -498,6 +574,17 @@
       <x:c r="Q3" s="12" t="str">
         <x:v>sim</x:v>
       </x:c>
+      <x:c r="R3" s="30" t="str"/>
+      <x:c r="S3" s="30" t="str"/>
+      <x:c r="T3" s="30" t="str"/>
+      <x:c r="U3" s="30" t="str"/>
+      <x:c r="V3" s="30" t="str"/>
+      <x:c r="W3" s="30" t="str"/>
+      <x:c r="X3" s="30" t="str"/>
+      <x:c r="Y3" s="30" t="str"/>
+      <x:c r="Z3" s="30" t="str"/>
+      <x:c r="AA3" s="30" t="str"/>
+      <x:c r="AB3" s="30" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -600,6 +687,14 @@
         <x:v>A importacao nao inclui ficheiros MP3 nem outros audios.</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>As colunas cifra_refrao e cifra_1 a cifra_10 sao opcionais.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>

</xml_diff>